<commit_message>
Refactor with CWL custom merchant trait update
</commit_message>
<xml_diff>
--- a/LangMod/CN/SourcePod.xlsx
+++ b/LangMod/CN/SourcePod.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="91">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -222,10 +222,10 @@
     <t xml:space="preserve">Friend</t>
   </si>
   <si>
-    <t xml:space="preserve">neutral,addStock,addZone_Kapul,addZone_TinkerCamp,addZone_Olvina,addZone_Aquli,addZone_Yowyn,addZone_Specwing,addZone_Mifu,addZone_Nefu,addZone_Palmia,addZone_Lothria,addZone_Mysilia,addZone_Derphy,addZone_Lumiest,addZone_Noyel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Merchant</t>
+    <t xml:space="preserve">neutral,addZone_Kapul,addZone_TinkerCamp,addZone_Olvina,addZone_Aquli,addZone_Yowyn,addZone_Specwing,addZone_Mifu,addZone_Nefu,addZone_Palmia,addZone_Lothria,addZone_Mysilia,addZone_Derphy,addZone_Lumiest,addZone_Noyel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OmegaMerchantPod042</t>
   </si>
   <si>
     <t xml:space="preserve">metal</t>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t xml:space="preserve">装甲商人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OmegaMerchantPod153</t>
   </si>
   <si>
     <t xml:space="preserve">f</t>
@@ -1327,7 +1330,7 @@
         <v>65</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="W5" s="1" t="s">
         <v>67</v>
@@ -1342,7 +1345,7 @@
         <v>70</v>
       </c>
       <c r="AN5" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AR5" s="1" t="s">
         <v>72</v>
@@ -1394,34 +1397,34 @@
         <v>33</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1477,34 +1480,34 @@
         <v>72</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="L4" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1048302" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>